<commit_message>
Document auto author sync in db_updater README + load .env.live in tunnel helper
- README: clarify that run_master_site_sync.py already fetches author_id/name; sync_wp_authors.py is only for re-syncs
- ssh_tunnel_helper: auto-load all env vars from .env.live (e.g. WP_CREDENTIAL_ENCRYPTION_KEY) so dev scripts work without manual export
- master_site_file: add new site entry

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portal_backend/scripts/db_updater/master_site_info/master_site_file.xlsx
+++ b/portal_backend/scripts/db_updater/master_site_info/master_site_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adil/Projects/Elci/doc_converter_service/portal_backend/scripts/db_updater/master_site_info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D96BCD33-AC65-FD40-A7AC-EDC305E287D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36635A3C-45B8-AB4C-AC2D-BEE00391B775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="18760" xr2:uid="{F15F579C-1C8E-9F41-8077-01E0A300B3F9}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19800" xr2:uid="{F15F579C-1C8E-9F41-8077-01E0A300B3F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="333">
   <si>
     <t>name</t>
   </si>
@@ -1023,6 +1023,18 @@
   </si>
   <si>
     <t>wp_admin_password</t>
+  </si>
+  <si>
+    <t>Apfelwelten.de</t>
+  </si>
+  <si>
+    <t>https://apfelwelten.de</t>
+  </si>
+  <si>
+    <t>Info@leventelci.de</t>
+  </si>
+  <si>
+    <t>BMSm FK9y 1J46 CAVa QxzU SAiv</t>
   </si>
 </sst>
 </file>
@@ -4418,49 +4430,66 @@
       </c>
     </row>
     <row r="95" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>330</v>
+      </c>
       <c r="C95" s="3" t="s">
         <v>172</v>
       </c>
+      <c r="D95" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="J95" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="L95" s="1" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="96" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="C96" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C96" s="3"/>
     </row>
     <row r="97" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C97" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C97" s="3"/>
     </row>
     <row r="98" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C98" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C98" s="3"/>
     </row>
     <row r="99" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C99" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C99" s="3"/>
     </row>
     <row r="100" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C100" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C100" s="3"/>
     </row>
     <row r="101" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C101" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C101" s="3"/>
     </row>
     <row r="102" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C102" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C102" s="3"/>
     </row>
     <row r="103" spans="3:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C103" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="C103" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>